<commit_message>
LBP standard correction to ng/ml
</commit_message>
<xml_diff>
--- a/LBP/standard/standard_lbp.xlsx
+++ b/LBP/standard/standard_lbp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brian\Desktop\zivkovic_lab\fiber_study\LBP\standard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BH\Desktop\HDL\Eddie\fiber_study\LBP\standard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A9566EE-6AAF-4CEF-ABD1-6525B40A8FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D3B833E-1BB2-424E-B60E-38C2E85B043E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{116D2DFF-6977-4112-8AF0-C3736CFD7AD6}"/>
+    <workbookView xWindow="-260" yWindow="0" windowWidth="8530" windowHeight="10200" xr2:uid="{116D2DFF-6977-4112-8AF0-C3736CFD7AD6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,9 +38,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
-    <t>conc_pg_ml</t>
-  </si>
-  <si>
     <t>S1</t>
   </si>
   <si>
@@ -66,6 +63,9 @@
   </si>
   <si>
     <t>sample</t>
+  </si>
+  <si>
+    <t>conc_ng_ml</t>
   </si>
 </sst>
 </file>
@@ -418,78 +418,78 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58495479-1214-49FF-A33F-87D13234EB0C}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" t="s">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
-      <c r="A2" t="s">
-        <v>1</v>
       </c>
       <c r="B2">
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4">
         <v>12.5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5">
         <v>6.25</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6">
         <v>3.125</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7">
         <v>1.5625</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8">
         <v>0.78129999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9">
         <v>0</v>

</xml_diff>